<commit_message>
Clarify B2 warmup and 34-month data scope
</commit_message>
<xml_diff>
--- a/docs/stock_automl_runs/20261018_b2_full_replay/B2四K全年复核_总体逐月每日逐笔.xlsx
+++ b/docs/stock_automl_runs/20261018_b2_full_replay/B2四K全年复核_总体逐月每日逐笔.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总体与逐月" sheetId="1" r:id="R7ed48cd2af854b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易逐笔" sheetId="2" r:id="R64ec4fdd0d0c4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日资金" sheetId="3" r:id="R147d97b9b4684899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三名候选" sheetId="4" r:id="Re0e2d31445ec4785"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则说明" sheetId="5" r:id="R48d3500d34ff4cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总体与逐月" sheetId="1" r:id="R400bae347d904893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易逐笔" sheetId="2" r:id="R7286337969ab4e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日资金" sheetId="3" r:id="R1488cfcfe2dc4f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三名候选" sheetId="4" r:id="Rc27511261b3c40ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则说明" sheetId="5" r:id="Rf093d27a13ee4495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月份范围" sheetId="6" r:id="R8e58107b56484b31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +23,7 @@
     <x:numFmt numFmtId="201" formatCode="@"/>
     <x:numFmt numFmtId="202" formatCode="0.0000;[Red](0.0000);–"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -78,8 +79,14 @@
       <x:color rgb="FF546779"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +96,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF203B59"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF4"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -129,7 +146,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -149,6 +166,10 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -453,7 +474,7 @@
     </x:row>
     <x:row r="2" ht="29" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>全年分钟数据已核验；B2同口径收益覆盖18个月。逐笔、每日与候选见后续页。</x:v>
+        <x:v>34个月原始范围＝16个月预热＋17个完整回测月＋1个未完回测月；月序对应见「月份范围」。</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1201,7 +1222,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84c410a4b73d401e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd17bcd12fdbe4a0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11261,7 +11282,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb20ee05a22164ce8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ce43e1337284dcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23399,7 +23420,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf341ad35bcee4adb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb528feff3cea4ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -61662,7 +61683,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4df03f8e22fc4c8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R193682c95dcb488c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -61766,4 +61787,491 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="20" t="str">
+        <x:v>B2四K｜34个月原始范围与18个月回测</x:v>
+      </x:c>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+    </x:row>
+    <x:row r="2" ht="31" customHeight="1">
+      <x:c r="A2" t="str">
+        <x:v>两轮各8个月预热；收益月序1—18对应全部月序17—34。最后一月尚未结束。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1"/>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="22" t="str">
+        <x:v>全部月序</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>阶段</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>收益月序</x:v>
+      </x:c>
+      <x:c r="D4" s="22" t="str">
+        <x:v>完整月</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C5" s="17"/>
+      <x:c r="D5" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C6" s="17"/>
+      <x:c r="D6" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C7" s="17"/>
+      <x:c r="D7" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C8" s="17"/>
+      <x:c r="D8" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C9" s="17"/>
+      <x:c r="D9" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C10" s="17"/>
+      <x:c r="D10" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="17" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>日线排序预热</x:v>
+      </x:c>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C13" s="17"/>
+      <x:c r="D13" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C14" s="17"/>
+      <x:c r="D14" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C15" s="17"/>
+      <x:c r="D15" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C16" s="17"/>
+      <x:c r="D16" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="17" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C17" s="17"/>
+      <x:c r="D17" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="17" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C18" s="17"/>
+      <x:c r="D18" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="17" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C19" s="17"/>
+      <x:c r="D19" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="17" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B20" s="17" t="str">
+        <x:v>四K规则预热</x:v>
+      </x:c>
+      <x:c r="C20" s="17"/>
+      <x:c r="D20" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="17" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B21" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="17" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B22" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C22" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="17" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B23" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C23" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D23" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="17" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B24" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C24" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D24" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="17" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C25" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="17" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B26" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C26" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D26" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="17" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B27" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C27" s="17" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D27" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="17" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B28" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C28" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D28" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="17" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B29" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C29" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D29" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="17" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B30" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C30" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D30" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="17" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C31" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D31" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="17" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B32" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C32" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D32" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="17" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B33" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C33" s="17" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D33" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="17" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B34" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C34" s="17" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D34" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="17" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B35" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C35" s="17" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D35" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="17" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B36" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D36" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="17" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B37" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C37" s="17" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D37" s="17" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="17" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B38" s="17" t="str">
+        <x:v>同口径回测</x:v>
+      </x:c>
+      <x:c r="C38" s="17" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D38" s="17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>